<commit_message>
feat(QA-5687): E2E test-recepcion pendientes acuse y rechazo
Add Cucumber scenarios TC-INT-017/018 chaining POST test-recepcion,
GET pendientes-recepcion and PUT acuse-recibo (accept/reject).

Includes probe script, npm scripts for E2E and full card closure,
and updated matriz/evidencias generators.

Co-authored-by: JFCandia-Digital <JFCandia-Digital@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/api-v3.5/matriz_api_test_recepcion_integracion_DocDigital.xlsx
+++ b/docs/api-v3.5/matriz_api_test_recepcion_integracion_DocDigital.xlsx
@@ -1731,7 +1731,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>POST /pruebas-integracion/comunicaciones/test-recepcion 200 | GET /comunicaciones/pendientes-recepcion?materia=... | PUT /comunicaciones/{id}/recepcion/{tareaId}/acuse-recibo</t>
+          <t>POST /pruebas-integracion/comunicaciones/test-recepcion 200 | GET /comunicaciones/pendientes-recepcion?materia=... | PUT /comunicaciones/{id}/recepcion/{tareaId}/acuse-recibo (isRechazada: false)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Pendiente ejecución</t>
+          <t>Pendiente ejecución — postTestRecepcionE2E.feature @TestRecepcion_E2E_Acuse</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Cucumber E2E; reports/index.html; features pendientes + acuse existentes</t>
+          <t>Cucumber @TestRecepcion_E2E_Acuse; reports/index.html</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>POST /pruebas-integracion/comunicaciones/test-recepcion 200 | GET pendientes-recepcion | PUT acuse-recibo con decisión rechazo</t>
+          <t>POST /pruebas-integracion/comunicaciones/test-recepcion 200 | GET pendientes-recepcion | PUT acuse-recibo con isRechazada: true</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Pendiente ejecución</t>
+          <t>Pendiente ejecución — postTestRecepcionE2E.feature @TestRecepcion_E2E_Rechazo</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Cucumber E2E; putAcuseRecibo.feature</t>
+          <t>Cucumber @TestRecepcion_E2E_Rechazo; reports/index.html</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">

</xml_diff>